<commit_message>
Update AIP retail petrol state prices
</commit_message>
<xml_diff>
--- a/data/petrol_state_weekly_prices.xlsx
+++ b/data/petrol_state_weekly_prices.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2149,6 +2149,35 @@
         <v>209.1</v>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B60" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="C60" t="n">
+        <v>211</v>
+      </c>
+      <c r="D60" t="n">
+        <v>209.8</v>
+      </c>
+      <c r="E60" t="n">
+        <v>212.6</v>
+      </c>
+      <c r="F60" t="n">
+        <v>208.5</v>
+      </c>
+      <c r="G60" t="n">
+        <v>211.3</v>
+      </c>
+      <c r="H60" t="n">
+        <v>232.4</v>
+      </c>
+      <c r="I60" t="n">
+        <v>215</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>